<commit_message>
Update Russia sheet Logo URL: 200 official logo URLs found from sites directly
Co-authored-by: Machibo <Machibo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/СМИ_карточки_для_сайта.xlsx
+++ b/СМИ_карточки_для_сайта.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/srrb.ru</t>
+          <t>https://srrb.ru/apple-touch-icon.png</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/apni.ru</t>
+          <t>https://apni.ru/uploads/Logo.svg</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/tvkinoradio.ru</t>
+          <t>https://tvkinoradio.ru/img/logo/tvkinoradio.png</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/politnavigator.net</t>
+          <t>https://www.politnavigator.net/wp-content/themes/politnav-puzzle/images/pnlogo.png</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/bloknot.ru</t>
+          <t>https://bloknot.ru/static/images/logo_color3.png</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/delovoymir.biz</t>
+          <t>https://region.center/data/moduleslogos/ac5557cf56c5ab10d8b525864891e909.png</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/business-magazine.online</t>
+          <t>https://region.center/data/moduleslogos/f339af0da3f8d6b5a8da975d0ace7c62.svg</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/garant.ru</t>
+          <t>https://www.garant.ru/static/www/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/prophotos.ru</t>
+          <t>https://my.prophotos.ru/assets/logo_prophotos_big-e2a018230a87b9724c0abdf904d49c3eec5d3dcd4d221a7af7207022b2b98c81.png</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/peopletalk.ru</t>
+          <t>https://peopletalk.ru/wp-content/themes/peopletalk2019/dist/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/versia.ru</t>
+          <t>https://versia.ru/images/newspaper.png</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/infox.ru</t>
+          <t>https://www.infox.ru/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/samag.ru</t>
+          <t>https://www.samag.ru/img/logo.jpg</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/itweek.ru</t>
+          <t>https://www.itweek.ru/images/itweek/logo.png</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/1sept.ru</t>
+          <t>https://1sept.ru/theme/logo.svg</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/finversia.ru</t>
+          <t>https://finversia.ru/site/themes/lapuzzle/images/header/Header_Logo.svg</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mir24.tv</t>
+          <t>https://images.mir24.tv/jzZtwM40HO2JiUckYTI5gRZ-PCCVCb3RBK_sOV818Dc/czM6Ly9taXIyNC10di9tZWRpYS9TZXR0aW5nc0xvZ28vaW1hZ2UvYWQ1ZTVmODItNWEyNS00MDVlLWIxYmItOTVmODlmMTZiMzY5L2xvZ29GLnN2Zw.svg</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/lenta.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/01/Lenta.svg</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/7days.ru</t>
+          <t>https://cdn.7days.ru/bitrix/templates/7days-redesign-2021/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vokrug.tv</t>
+          <t>https://www.vokrug.tv/images/logo-new.svg</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/fedpress.ru</t>
+          <t>https://fedpress.ru/themes/fp/images/main/logo-text.png</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/securitylab.ru</t>
+          <t>https://www.securitylab.ru/img/logo/logo-header.svg</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/osnmedia.ru</t>
+          <t>https://www.osnmedia.ru/wp-content/uploads/2025/05/logo-new-light.png</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/snob.ru</t>
+          <t>https://snob.ru/apple-touch-icon.png</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/comnews.ru</t>
+          <t>https://www.comnews.ru/themes/site/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/tproger.ru</t>
+          <t>https://tproger.ru/images/favicons/favicon.svg</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/cnews.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/07/CNews_logo.svg</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/iz.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4d/Izvestia.svg</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sport-express.ru</t>
+          <t>https://ss.sport-express.net/fb/img/icons/logos/se-logo.svg</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/newdaynews.ru</t>
+          <t>https://newdaynews.ru/global/flb/newdaynews.logo.svg</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/gazetametro.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5f/Metro_International_Logo.svg</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/5-tv.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/c0/5-tv_logo_%282023%29.svg</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/dk.ru</t>
+          <t>https://www.dk.ru/assets/logo_dk-756cff44c32801053911cb9f9243f9c8.svg</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/strategyjournal.ru</t>
+          <t>https://strategyjournal.ru/wp-content/themes/strategyjournal/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/retailer.ru</t>
+          <t>https://retailer.ru/wp-content/themes/monstroid2/assets/images/retailer-logo.svg</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mk.ru</t>
+          <t>https://www.mk.ru/media/mkru2020/img/mk-logo.svg</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/aif.ru</t>
+          <t>https://aif.ru/redesign2018/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vedomosti.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/0c/Vedomosti_logo.svg</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ng.ru</t>
+          <t>https://www.ng.ru/bitrix/templates/ng/i/logo.png</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/business.ru</t>
+          <t>https://www.business.ru/themes/business_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kom-dir.ru</t>
+          <t>https://www.kom-dir.ru/themes/kom-dir_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/glavbukh.ru</t>
+          <t>https://www.glavbukh.ru/themes/glavbukh_ru/assets/frontend/images/logo_red.svg</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/26-2.ru</t>
+          <t>https://www.26-2.ru/themes/26-2_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/buhsoft.ru</t>
+          <t>https://www.buhsoft.ru/themes/buhsoft_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/pro-personal.ru</t>
+          <t>https://www.pro-personal.ru/themes/pro-personal_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kdelo.ru</t>
+          <t>https://www.kdelo.ru/themes/kdelo_ru/assets/frontend/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/tass.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/95/TASS_Logo_%28Latin%29_2022.svg</t>
         </is>
       </c>
     </row>
@@ -3753,7 +3753,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/gazeta.ru</t>
+          <t>https://static.gazeta.ru/nm2015/i/logo_gazeta.svg</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vm.ru</t>
+          <t>https://vm.ru/img/main_logo.svg</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/news.ru</t>
+          <t>https://news.ru/assets/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/profile.ru</t>
+          <t>https://cdn.profile.ru/wp-content/themes/profile/assets/img/profile-logo-delovoy.svg</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/oilcapital.ru</t>
+          <t>https://oilcapital.ru/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/business-gazeta.ru</t>
+          <t>https://business-gazeta.ru/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ko.ru</t>
+          <t>https://ko.ru/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/dp.ru</t>
+          <t>https://www.dp.ru/assets/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/popmech.ru</t>
+          <t>https://popmech.ru/_nuxt/img/logo-techinsider-full_2203343.svg</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/svpressa.ru</t>
+          <t>https://svpressa.ru/i/logo-svpressa.svg</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ridus.ru</t>
+          <t>https://www.ridus.ru/_images/logo.png</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/dni.ru</t>
+          <t>https://dni.ru/static/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/utro.ru</t>
+          <t>https://utro.ru/static/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kleo.ru</t>
+          <t>https://www.kleo.ru/wp-content/uploads/2026/01/kleo-logo.svg</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/newizv.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/15/%D0%9D%D0%98_%D0%BB%D0%BE%D0%B3%D0%BE.png</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/rosbalt.ru</t>
+          <t>https://www.rosbalt.ru/img/icons/icon-512x512.png</t>
         </is>
       </c>
     </row>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/monocle.ru</t>
+          <t>https://monocle.ru/static/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/rg.ru</t>
+          <t>https://cdnstatic.rg.ru/svg/touch-icon.svg</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/runews24.ru</t>
+          <t>https://runews24.ru/assets/images/logo2.png</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/angi.ru</t>
+          <t>https://www.angi.ru/images/homepage.png</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/naked-science.ru</t>
+          <t>https://naked-science.ru/assets/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/globalcio.ru</t>
+          <t>https://globalcio.ru/local/static/html/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/businesstory.ru</t>
+          <t>https://businesstory.ru/wp-content/uploads/2026/05/bs-logo.png</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ict-online.ru</t>
+          <t>https://www.ict-online.ru/old/gif/max_mess_logo.svg</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/logirus.ru</t>
+          <t>https://logirus.ru/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/24gadget.ru</t>
+          <t>https://24gadget.ru/templates/Default/images/new/logo_s.gif</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/marieclaire.com</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/d0/Marie_Claire_Magazine_logo.svg</t>
         </is>
       </c>
     </row>
@@ -5562,7 +5562,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/3dnews.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4b/3DNews_logo.svg</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/servernews.ru</t>
+          <t>https://servernews.ru/assets/external/servernews.ru/images/logo.jpg</t>
         </is>
       </c>
     </row>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/new-retail.ru</t>
+          <t>https://new-retail.ru/img/logo/logo.png</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/nakanune.ru</t>
+          <t>https://media.nakanune.ru/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/telecomdaily.ru</t>
+          <t>https://telecomdaily.ru/faaf6981f14537b11b8277d64fabc69f.png</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/bigpicture.ru</t>
+          <t>https://bigpicture.ru/wp-content/themes/bigpicture-new/assets/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kommersant.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/8c/Logo_Kommersant.svg</t>
         </is>
       </c>
     </row>
@@ -6031,7 +6031,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/eadaily.com</t>
+          <t>https://static1.eadaily.com/i/logos/logo-squared-400.png</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sostav.ru</t>
+          <t>https://www.sostav.ru/app/public/design/logo2918-05v3.svg</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ura.news</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/69/URA.RU_logo.svg</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/seonews.ru</t>
+          <t>https://www.seonews.ru/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/likeni.ru</t>
+          <t>https://www.likeni.ru/assets/img/logo-mini.png</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/life.ru</t>
+          <t>https://life.ru/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/omanhit.ru</t>
+          <t>https://www.womanhit.ru/static/images/og/womanhit_ru_og_logo_1200_720.png</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/avtovzglyad.ru</t>
+          <t>https://www.avtovzglyad.ru/static/images/avtovzglyad-logo.svg</t>
         </is>
       </c>
     </row>
@@ -6634,7 +6634,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ohotniki.ru</t>
+          <t>https://www.ohotniki.ru/static/images/ohotniki-logo.svg</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mperspektiva.ru</t>
+          <t>https://mperspektiva.ru/local/templates/mp/s/images/tmp_file/header/dec-logo.webp</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/beautyhack.ru</t>
+          <t>https://beautyhack.ru/assets/images/logo2.png</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6835,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sobaka.ru</t>
+          <t>https://www.sobaka.ru/img/sobaka.svg</t>
         </is>
       </c>
     </row>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sobaka.ru</t>
+          <t>https://www.sobaka.ru/img/sobaka.svg</t>
         </is>
       </c>
     </row>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sobaka.ru</t>
+          <t>https://www.sobaka.ru/img/sobaka.svg</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/forbes.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/db/Forbes_logo.svg</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/stroygaz.ru</t>
+          <t>https://stroygaz.ru/upload/uf/e61/oekrgwiovsiba5ajvv6147lsauedss2g.webp</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/regnum.ru</t>
+          <t>https://regnum.ru/main_logo.svg</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/topcor.ru</t>
+          <t>https://topcor.ru/templates/topcor/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sfera.fm</t>
+          <t>https://sfera.fm/assets/media/logo/logo_sfera_header.png</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7371,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/brl.mk.ru</t>
+          <t>https://brl.mk.ru/media/mkru2020/img/mk-logo.svg</t>
         </is>
       </c>
     </row>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/novate.ru</t>
+          <t>https://novate.ru/img/logo.svg</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/beautycarteblanche.ru</t>
+          <t>https://static.tildacdn.com/tild3930-3036-4536-a464-363733353938/BCB_logo_1.svg</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vokrug.tv</t>
+          <t>https://www.vokrug.tv/images/logo-new.svg</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vokrugsveta.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/vokrugsveta/8b7f3beb.svg</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/oman.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/woman/2cb6624f.svg</t>
         </is>
       </c>
     </row>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/day.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/wday/2cb6624f.svg</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7840,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/thegirl.ru</t>
+          <t>https://thegirl.ru/public/sprites/thegirl/e5cb1e72ce8b.svg</t>
         </is>
       </c>
     </row>
@@ -7907,7 +7907,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/starhit.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/starhit/500f077c.svg</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/parents.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/parents/b1a1d258.svg</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8041,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mydecor.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/mcmaison/2cb6624f.svg</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/doctorpiter.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/doctorpiter/e4197781.svg</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/the-day.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/wday/2cb6624f.svg</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/maximonline.ru</t>
+          <t>https://cdn.hsmedia.ru/dist/maxim/f8d1d209.svg</t>
         </is>
       </c>
     </row>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/psychologies.ru</t>
+          <t>https://cdn.hsmedia.ru/ump-webapp-public/dist/client/assets/psychologies_lg_bg-light-DG40Nryg.svg</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8376,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/fashiontime.ru</t>
+          <t>https://www.fashiontime.ru/bitrix/templates/ft.v3/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -8443,7 +8443,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/oane.ws</t>
+          <t>https://oane.ws/templates/oane_new/logo-old.png</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/terrnews.com</t>
+          <t>https://terrnews.com/templates/Hint-utf8/images/logo66.png</t>
         </is>
       </c>
     </row>
@@ -8577,7 +8577,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kadara.ru</t>
+          <t>https://kadara.ru/wp-content/uploads/2019/12/kadara-logo.png</t>
         </is>
       </c>
     </row>
@@ -8644,7 +8644,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/monavista.ru</t>
+          <t>https://monavista.ru/templates/newshub/images/logo-old.png</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/vestnik.net</t>
+          <t>https://vestnik.net/images/logo_in_html.png</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/nvspost.ru</t>
+          <t>https://nvspost.ru/templates/lifewatcher/images/logo3.png</t>
         </is>
       </c>
     </row>
@@ -8845,7 +8845,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/spb.kp.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/68/K_Pravda_Logo_Modern.svg</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/belarus.kp.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/68/K_Pravda_Logo_Modern.svg</t>
         </is>
       </c>
     </row>
@@ -9046,7 +9046,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/news-24.ru</t>
+          <t>https://news-24.ru/wp-content/uploads/2025/01/logon24.png</t>
         </is>
       </c>
     </row>
@@ -9113,7 +9113,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/smi24.news</t>
+          <t>https://smi24.news/wp-content/uploads/2024/12/group-158-1.svg</t>
         </is>
       </c>
     </row>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/frequentflyers.ru</t>
+          <t>https://www.frequentflyers.ru/wp-content/uploads/2015/10/fflogo6.png</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9649,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/adindex.ru</t>
+          <t>https://adindex.ru/assets/img/logo-adindex.svg</t>
         </is>
       </c>
     </row>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/artagmag.ru</t>
+          <t>https://static.tildacdn.com/tild3938-6436-4639-b565-343838653436/Logo.svg</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sport24.ru</t>
+          <t>https://img.artlebedev.ru/everything/sport24/identity/media/icons/s24_port.svg</t>
         </is>
       </c>
     </row>
@@ -9850,7 +9850,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/prufy.ru</t>
+          <t>https://prufy.ru/images/reg/prufy.ru.svg</t>
         </is>
       </c>
     </row>
@@ -9984,7 +9984,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/moneytimes.ru</t>
+          <t>https://www.moneytimes.ru/images/moneytimes-logo.png</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/english.pravda.ru</t>
+          <t>https://english.pravda.ru/pix/logo_white.png</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10118,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/medpulse.ru</t>
+          <t>https://www.medpulse.ru/image/upload/logo512.jpg</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/newsinfo.ru</t>
+          <t>https://www.newsinfo.ru/images/newsinfo-logo.png</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/politonline.ru</t>
+          <t>https://www.politonline.ru/assets/logo-5-4679515ece2fdfeb4567553a15565643.png</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/yoki.ru</t>
+          <t>https://www.yoki.ru/images/yoki-logo.png</t>
         </is>
       </c>
     </row>
@@ -10453,7 +10453,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ecosever.ru</t>
+          <t>https://www.ecosever.ru/images/ecosever-logo.png</t>
         </is>
       </c>
     </row>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/nationaljournal.ru</t>
+          <t>https://www.nationaljournal.ru/pix/nationaljournal-logo.png</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/rusday.com</t>
+          <t>https://www.rusday.com/pix/rusday-logo.png</t>
         </is>
       </c>
     </row>
@@ -10654,7 +10654,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/electorat.info</t>
+          <t>https://www.electorat.info/pix/electorat-logo.png</t>
         </is>
       </c>
     </row>
@@ -10721,7 +10721,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mostimes.com</t>
+          <t>https://www.mostimes.com/images/mostimes-logo.png</t>
         </is>
       </c>
     </row>
@@ -10788,7 +10788,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/pora.ru</t>
+          <t>https://www.pora.ru/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/glavtema.ru</t>
+          <t>https://www.glavtema.ru/pix/glavtema-logo.png</t>
         </is>
       </c>
     </row>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/prbn.ru</t>
+          <t>https://www.prbn.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/bigness.ru</t>
+          <t>https://www.bigness.ru/pix/logo.gif</t>
         </is>
       </c>
     </row>
@@ -11056,7 +11056,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/militarytimes.ru</t>
+          <t>https://www.militarytimes.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11123,7 +11123,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/fizcultprivet.ru</t>
+          <t>https://www.fizcultprivet.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11190,7 +11190,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/poplawok.ru</t>
+          <t>https://www.poplawok.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/autokolonka.ru</t>
+          <t>https://www.autokolonka.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11324,7 +11324,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/repairshome.ru</t>
+          <t>https://www.repairshome.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11391,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/dailyshow.ru</t>
+          <t>https://www.dailyshow.ru/images/dailyshow-logo.gif</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/missus.ru</t>
+          <t>https://www.missus.ru/pix/logo.gif</t>
         </is>
       </c>
     </row>
@@ -11525,7 +11525,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/bigcaucasus.com</t>
+          <t>https://www.bigcaucasus.com/pix/smalllogo.jpg</t>
         </is>
       </c>
     </row>
@@ -11592,7 +11592,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/georgiatimes.info</t>
+          <t>https://www.georgiatimes.info/images/georgiatimes-logo.jpg</t>
         </is>
       </c>
     </row>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/pravda.ru</t>
+          <t>https://www.pravda.ru/pix/logo600_60.png</t>
         </is>
       </c>
     </row>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/aviation21.ru</t>
+          <t>https://aviation21.ru/wp-content/uploads/2017/03/logo-1.png</t>
         </is>
       </c>
     </row>
@@ -11860,7 +11860,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/asninfo.ru</t>
+          <t>https://asninfo.ru/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/78.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/2/24/TV78logo.svg</t>
         </is>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/thevoicemag.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/67/Logo_of_Russian_magazine_The_Voice.svg</t>
         </is>
       </c>
     </row>
@@ -12061,7 +12061,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/moskvichmag.ru</t>
+          <t>https://moskvichmag.ru/wp-content/themes/moskmag-new/assets/img/svg/mm-xl-logo.svg</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/rbc.ru</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/f1/RBK_logo.svg</t>
         </is>
       </c>
     </row>
@@ -12195,7 +12195,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/moslenta.ru</t>
+          <t>https://moslenta.ru/favicon.svg</t>
         </is>
       </c>
     </row>
@@ -12262,7 +12262,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/kapital.kz</t>
+          <t>https://kapital.kz/logo.png</t>
         </is>
       </c>
     </row>
@@ -12329,7 +12329,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/lsm.kz</t>
+          <t>https://lsm.kz/static/img/logo.png</t>
         </is>
       </c>
     </row>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/newsmaker.md</t>
+          <t>https://newsmaker.md/wp-content/uploads/2019/01/logo_square.jpg</t>
         </is>
       </c>
     </row>
@@ -12463,7 +12463,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/akipress.org</t>
+          <t>https://cdn-1.aki.kg/st_akipress/logo_wide_300x48.png</t>
         </is>
       </c>
     </row>
@@ -12530,7 +12530,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/24.kg</t>
+          <t>https://24.kg/assets/39aedacb/images/logo.png</t>
         </is>
       </c>
     </row>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/noi.md</t>
+          <t>https://noi.md/images/logo_noi_blue.jpg</t>
         </is>
       </c>
     </row>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/uzdaily.uz</t>
+          <t>https://www.uzdaily.uz/static/web/files/logo.258d31191858.svg</t>
         </is>
       </c>
     </row>
@@ -12731,7 +12731,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/inform.kz</t>
+          <t>https://www.inform.kz/static/img/favicon.svg</t>
         </is>
       </c>
     </row>
@@ -12798,7 +12798,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/remedium.ru</t>
+          <t>https://remedium.ru/upload/medialibrary/43b/Remedium-logo-2019-MAIN.png</t>
         </is>
       </c>
     </row>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/medvestnik.ru</t>
+          <t>https://medvestnik.ru/apps/mv/assets/cache/images/c7aa52eecd.svg</t>
         </is>
       </c>
     </row>
@@ -12932,7 +12932,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/incrussia.ru</t>
+          <t>https://incrussia.ru/wp-content/themes/inc/img/ink_logo_space.svg</t>
         </is>
       </c>
     </row>
@@ -12999,7 +12999,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/apptractor.ru</t>
+          <t>https://apptractor.ru/wp-content/uploads/2025/10/logowebp-1.webp</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/investfuture.ru</t>
+          <t>https://investfuture.ru/static/logo.png</t>
         </is>
       </c>
     </row>
@@ -13133,7 +13133,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/onliner.by</t>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/f3/Logo-onliner-by.png</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13200,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/bits.media</t>
+          <t>https://bits.media/local/templates/bits.media/images/bits4.png</t>
         </is>
       </c>
     </row>
@@ -13267,7 +13267,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/telegraf.news</t>
+          <t>https://telegraf.news/_astro/logo_black.hKlVZoUa.svg</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/liter.kz</t>
+          <t>https://liter.kz/build/images/liter-logo-news.png</t>
         </is>
       </c>
     </row>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/orda.kz</t>
+          <t>https://orda.kz/img/logo_d.svg</t>
         </is>
       </c>
     </row>
@@ -13468,7 +13468,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/dcjournal.ru</t>
+          <t>https://dcjournal.ru/theme/codirf/images/h-logo6.png</t>
         </is>
       </c>
     </row>
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/telecombloger.ru</t>
+          <t>https://telecombloger.ru/wp-content/uploads/2024/12/Logo.png</t>
         </is>
       </c>
     </row>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/urbc.ru</t>
+          <t>https://urbc.ru/templates/Default/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/haqqin.az</t>
+          <t>https://upload.wikimedia.org/wikipedia/ru/9/9d/%D0%9B%D0%BE%D0%B3%D0%BE%D1%82%D0%B8%D0%BF_Haqqin.az.svg</t>
         </is>
       </c>
     </row>
@@ -13736,7 +13736,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mosregion.info</t>
+          <t>https://www.mosregion.info/wp-content/uploads/2024/09/mosregion_logo.png</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sila-rf.ru</t>
+          <t>https://www.sila-rf.ru/wp-content/uploads/2022/02/sila-rf.png</t>
         </is>
       </c>
     </row>
@@ -13870,7 +13870,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/sibmedia.ru</t>
+          <t>https://www.sibmedia.ru/wp-content/uploads/2024/07/sibmedia_logo.png</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ladys.media</t>
+          <t>https://www.ladys.media/wp-content/themes/ladys/images/logos/logo_desktop.svg</t>
         </is>
       </c>
     </row>
@@ -14004,7 +14004,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/socialinform.ru</t>
+          <t>https://www.socialinform.ru/wp-content/uploads/2024/02/socnews_logo-1.png</t>
         </is>
       </c>
     </row>
@@ -14071,7 +14071,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/myeconomy.ru</t>
+          <t>https://www.myeconomy.ru/wp-content/uploads/2024/11/economy-logo.png</t>
         </is>
       </c>
     </row>
@@ -14138,7 +14138,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/ecopravda.ru</t>
+          <t>https://www.ecopravda.ru/wp-content/uploads/2022/07/Group-210.jpg</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14205,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/medzdrav.info</t>
+          <t>https://medzdrav.info/wp-content/uploads/2024/01/logo_header.svg</t>
         </is>
       </c>
     </row>
@@ -14272,7 +14272,7 @@
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/today.ua</t>
+          <t>https://today.ua/svg/logo.svg</t>
         </is>
       </c>
     </row>
@@ -14339,7 +14339,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/beautyhunter.ru</t>
+          <t>https://beautyhunter.ru/attachments/Image/bhlogo36.png</t>
         </is>
       </c>
     </row>
@@ -14406,7 +14406,7 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/informator.ua</t>
+          <t>https://informator.ua/images/logo.svg</t>
         </is>
       </c>
     </row>
@@ -14473,7 +14473,7 @@
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/itechua.com</t>
+          <t>https://itechua.com/wp-content/uploads/2024/08/itechua-logo.png</t>
         </is>
       </c>
     </row>
@@ -14540,7 +14540,7 @@
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/mignews.ua</t>
+          <t>https://mignews.ua/static/img/logo_ua.png</t>
         </is>
       </c>
     </row>
@@ -14607,7 +14607,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/it-world.ru</t>
+          <t>https://www.it-world.ru/local/templates/.default/img/logo/logo_s1.svg</t>
         </is>
       </c>
     </row>
@@ -14675,7 +14675,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>https://logos.hunter.io/gazeta.ua</t>
+          <t>https://gazeta.ua/images/svg/gazeta.svg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert Logo URL to Hunter.io database (logos.hunter.io/{domain})
Co-authored-by: Machibo <Machibo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/СМИ_карточки_для_сайта.xlsx
+++ b/СМИ_карточки_для_сайта.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>https://srrb.ru/apple-touch-icon.png</t>
+          <t>https://logos.hunter.io/srrb.ru</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://apni.ru/uploads/Logo.svg</t>
+          <t>https://logos.hunter.io/apni.ru</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://tvkinoradio.ru/img/logo/tvkinoradio.png</t>
+          <t>https://logos.hunter.io/tvkinoradio.ru</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://www.politnavigator.net/wp-content/themes/politnav-puzzle/images/pnlogo.png</t>
+          <t>https://logos.hunter.io/politnavigator.net</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>https://bloknot.ru/static/images/logo_color3.png</t>
+          <t>https://logos.hunter.io/bloknot.ru</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>https://region.center/data/moduleslogos/ac5557cf56c5ab10d8b525864891e909.png</t>
+          <t>https://logos.hunter.io/delovoymir.biz</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://region.center/data/moduleslogos/f339af0da3f8d6b5a8da975d0ace7c62.svg</t>
+          <t>https://logos.hunter.io/business-magazine.online</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://www.garant.ru/static/www/img/logo.svg</t>
+          <t>https://logos.hunter.io/garant.ru</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://my.prophotos.ru/assets/logo_prophotos_big-e2a018230a87b9724c0abdf904d49c3eec5d3dcd4d221a7af7207022b2b98c81.png</t>
+          <t>https://logos.hunter.io/prophotos.ru</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://peopletalk.ru/wp-content/themes/peopletalk2019/dist/img/logo.svg</t>
+          <t>https://logos.hunter.io/peopletalk.ru</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://versia.ru/images/newspaper.png</t>
+          <t>https://logos.hunter.io/versia.ru</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://www.infox.ru/img/logo.png</t>
+          <t>https://logos.hunter.io/infox.ru</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://www.samag.ru/img/logo.jpg</t>
+          <t>https://logos.hunter.io/samag.ru</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>https://www.itweek.ru/images/itweek/logo.png</t>
+          <t>https://logos.hunter.io/itweek.ru</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://1sept.ru/theme/logo.svg</t>
+          <t>https://logos.hunter.io/1sept.ru</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://finversia.ru/site/themes/lapuzzle/images/header/Header_Logo.svg</t>
+          <t>https://logos.hunter.io/finversia.ru</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://images.mir24.tv/jzZtwM40HO2JiUckYTI5gRZ-PCCVCb3RBK_sOV818Dc/czM6Ly9taXIyNC10di9tZWRpYS9TZXR0aW5nc0xvZ28vaW1hZ2UvYWQ1ZTVmODItNWEyNS00MDVlLWIxYmItOTVmODlmMTZiMzY5L2xvZ29GLnN2Zw.svg</t>
+          <t>https://logos.hunter.io/mir24.tv</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/0/01/Lenta.svg</t>
+          <t>https://logos.hunter.io/lenta.ru</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://cdn.7days.ru/bitrix/templates/7days-redesign-2021/images/logo.svg</t>
+          <t>https://logos.hunter.io/7days.ru</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>https://www.vokrug.tv/images/logo-new.svg</t>
+          <t>https://logos.hunter.io/vokrug.tv</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>https://fedpress.ru/themes/fp/images/main/logo-text.png</t>
+          <t>https://logos.hunter.io/fedpress.ru</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>https://www.securitylab.ru/img/logo/logo-header.svg</t>
+          <t>https://logos.hunter.io/securitylab.ru</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>https://www.osnmedia.ru/wp-content/uploads/2025/05/logo-new-light.png</t>
+          <t>https://logos.hunter.io/osnmedia.ru</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>https://snob.ru/apple-touch-icon.png</t>
+          <t>https://logos.hunter.io/snob.ru</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>https://www.comnews.ru/themes/site/images/logo.png</t>
+          <t>https://logos.hunter.io/comnews.ru</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>https://tproger.ru/images/favicons/favicon.svg</t>
+          <t>https://logos.hunter.io/tproger.ru</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/0/07/CNews_logo.svg</t>
+          <t>https://logos.hunter.io/cnews.ru</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/4/4d/Izvestia.svg</t>
+          <t>https://logos.hunter.io/iz.ru</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>https://ss.sport-express.net/fb/img/icons/logos/se-logo.svg</t>
+          <t>https://logos.hunter.io/sport-express.ru</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>https://newdaynews.ru/global/flb/newdaynews.logo.svg</t>
+          <t>https://logos.hunter.io/newdaynews.ru</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/5/5f/Metro_International_Logo.svg</t>
+          <t>https://logos.hunter.io/gazetametro.ru</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/c/c0/5-tv_logo_%282023%29.svg</t>
+          <t>https://logos.hunter.io/5-tv.ru</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>https://www.dk.ru/assets/logo_dk-756cff44c32801053911cb9f9243f9c8.svg</t>
+          <t>https://logos.hunter.io/dk.ru</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>https://strategyjournal.ru/wp-content/themes/strategyjournal/img/logo.svg</t>
+          <t>https://logos.hunter.io/strategyjournal.ru</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>https://retailer.ru/wp-content/themes/monstroid2/assets/images/retailer-logo.svg</t>
+          <t>https://logos.hunter.io/retailer.ru</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>https://www.mk.ru/media/mkru2020/img/mk-logo.svg</t>
+          <t>https://logos.hunter.io/mk.ru</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>https://aif.ru/redesign2018/img/logo.svg</t>
+          <t>https://logos.hunter.io/aif.ru</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/0/0c/Vedomosti_logo.svg</t>
+          <t>https://logos.hunter.io/vedomosti.ru</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>https://www.ng.ru/bitrix/templates/ng/i/logo.png</t>
+          <t>https://logos.hunter.io/ng.ru</t>
         </is>
       </c>
     </row>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>https://www.business.ru/themes/business_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/business.ru</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>https://www.kom-dir.ru/themes/kom-dir_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/kom-dir.ru</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>https://www.glavbukh.ru/themes/glavbukh_ru/assets/frontend/images/logo_red.svg</t>
+          <t>https://logos.hunter.io/glavbukh.ru</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>https://www.26-2.ru/themes/26-2_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/26-2.ru</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>https://www.buhsoft.ru/themes/buhsoft_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/buhsoft.ru</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>https://www.pro-personal.ru/themes/pro-personal_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/pro-personal.ru</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>https://www.kdelo.ru/themes/kdelo_ru/assets/frontend/images/logo.png</t>
+          <t>https://logos.hunter.io/kdelo.ru</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/9/95/TASS_Logo_%28Latin%29_2022.svg</t>
+          <t>https://logos.hunter.io/tass.ru</t>
         </is>
       </c>
     </row>
@@ -3753,7 +3753,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>https://static.gazeta.ru/nm2015/i/logo_gazeta.svg</t>
+          <t>https://logos.hunter.io/gazeta.ru</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>https://vm.ru/img/main_logo.svg</t>
+          <t>https://logos.hunter.io/vm.ru</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>https://news.ru/assets/images/logo.svg</t>
+          <t>https://logos.hunter.io/news.ru</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://cdn.profile.ru/wp-content/themes/profile/assets/img/profile-logo-delovoy.svg</t>
+          <t>https://logos.hunter.io/profile.ru</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://oilcapital.ru/img/logo.svg</t>
+          <t>https://logos.hunter.io/oilcapital.ru</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://business-gazeta.ru/img/logo.svg</t>
+          <t>https://logos.hunter.io/business-gazeta.ru</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://ko.ru/img/logo.png</t>
+          <t>https://logos.hunter.io/ko.ru</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://www.dp.ru/assets/images/logo.png</t>
+          <t>https://logos.hunter.io/dp.ru</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://popmech.ru/_nuxt/img/logo-techinsider-full_2203343.svg</t>
+          <t>https://logos.hunter.io/popmech.ru</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://svpressa.ru/i/logo-svpressa.svg</t>
+          <t>https://logos.hunter.io/svpressa.ru</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://www.ridus.ru/_images/logo.png</t>
+          <t>https://logos.hunter.io/ridus.ru</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://dni.ru/static/img/logo.png</t>
+          <t>https://logos.hunter.io/dni.ru</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://utro.ru/static/img/logo.png</t>
+          <t>https://logos.hunter.io/utro.ru</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://www.kleo.ru/wp-content/uploads/2026/01/kleo-logo.svg</t>
+          <t>https://logos.hunter.io/kleo.ru</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/1/15/%D0%9D%D0%98_%D0%BB%D0%BE%D0%B3%D0%BE.png</t>
+          <t>https://logos.hunter.io/newizv.ru</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>https://www.rosbalt.ru/img/icons/icon-512x512.png</t>
+          <t>https://logos.hunter.io/rosbalt.ru</t>
         </is>
       </c>
     </row>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>https://monocle.ru/static/img/logo.svg</t>
+          <t>https://logos.hunter.io/monocle.ru</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>https://cdnstatic.rg.ru/svg/touch-icon.svg</t>
+          <t>https://logos.hunter.io/rg.ru</t>
         </is>
       </c>
     </row>
@@ -4959,7 +4959,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>https://runews24.ru/assets/images/logo2.png</t>
+          <t>https://logos.hunter.io/runews24.ru</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>https://www.angi.ru/images/homepage.png</t>
+          <t>https://logos.hunter.io/angi.ru</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>https://naked-science.ru/assets/images/logo.svg</t>
+          <t>https://logos.hunter.io/naked-science.ru</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>https://globalcio.ru/local/static/html/images/logo.svg</t>
+          <t>https://logos.hunter.io/globalcio.ru</t>
         </is>
       </c>
     </row>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>https://businesstory.ru/wp-content/uploads/2026/05/bs-logo.png</t>
+          <t>https://logos.hunter.io/businesstory.ru</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5294,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>https://www.ict-online.ru/old/gif/max_mess_logo.svg</t>
+          <t>https://logos.hunter.io/ict-online.ru</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>https://logirus.ru/img/logo.png</t>
+          <t>https://logos.hunter.io/logirus.ru</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>https://24gadget.ru/templates/Default/images/new/logo_s.gif</t>
+          <t>https://logos.hunter.io/24gadget.ru</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5495,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/d/d0/Marie_Claire_Magazine_logo.svg</t>
+          <t>https://logos.hunter.io/marieclaire.com</t>
         </is>
       </c>
     </row>
@@ -5562,7 +5562,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/4/4b/3DNews_logo.svg</t>
+          <t>https://logos.hunter.io/3dnews.ru</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>https://servernews.ru/assets/external/servernews.ru/images/logo.jpg</t>
+          <t>https://logos.hunter.io/servernews.ru</t>
         </is>
       </c>
     </row>
@@ -5696,7 +5696,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>https://new-retail.ru/img/logo/logo.png</t>
+          <t>https://logos.hunter.io/new-retail.ru</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>https://media.nakanune.ru/images/logo.png</t>
+          <t>https://logos.hunter.io/nakanune.ru</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>https://telecomdaily.ru/faaf6981f14537b11b8277d64fabc69f.png</t>
+          <t>https://logos.hunter.io/telecomdaily.ru</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>https://bigpicture.ru/wp-content/themes/bigpicture-new/assets/img/logo.svg</t>
+          <t>https://logos.hunter.io/bigpicture.ru</t>
         </is>
       </c>
     </row>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/8/8c/Logo_Kommersant.svg</t>
+          <t>https://logos.hunter.io/kommersant.ru</t>
         </is>
       </c>
     </row>
@@ -6031,7 +6031,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>https://static1.eadaily.com/i/logos/logo-squared-400.png</t>
+          <t>https://logos.hunter.io/eadaily.com</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>https://www.sostav.ru/app/public/design/logo2918-05v3.svg</t>
+          <t>https://logos.hunter.io/sostav.ru</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/6/69/URA.RU_logo.svg</t>
+          <t>https://logos.hunter.io/ura.news</t>
         </is>
       </c>
     </row>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>https://www.seonews.ru/images/logo.svg</t>
+          <t>https://logos.hunter.io/seonews.ru</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>https://www.likeni.ru/assets/img/logo-mini.png</t>
+          <t>https://logos.hunter.io/likeni.ru</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>https://life.ru/img/logo.png</t>
+          <t>https://logos.hunter.io/life.ru</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>https://www.womanhit.ru/static/images/og/womanhit_ru_og_logo_1200_720.png</t>
+          <t>https://logos.hunter.io/omanhit.ru</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>https://www.avtovzglyad.ru/static/images/avtovzglyad-logo.svg</t>
+          <t>https://logos.hunter.io/avtovzglyad.ru</t>
         </is>
       </c>
     </row>
@@ -6634,7 +6634,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>https://www.ohotniki.ru/static/images/ohotniki-logo.svg</t>
+          <t>https://logos.hunter.io/ohotniki.ru</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>https://mperspektiva.ru/local/templates/mp/s/images/tmp_file/header/dec-logo.webp</t>
+          <t>https://logos.hunter.io/mperspektiva.ru</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6768,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>https://beautyhack.ru/assets/images/logo2.png</t>
+          <t>https://logos.hunter.io/beautyhack.ru</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6835,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>https://www.sobaka.ru/img/sobaka.svg</t>
+          <t>https://logos.hunter.io/sobaka.ru</t>
         </is>
       </c>
     </row>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>https://www.sobaka.ru/img/sobaka.svg</t>
+          <t>https://logos.hunter.io/sobaka.ru</t>
         </is>
       </c>
     </row>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>https://www.sobaka.ru/img/sobaka.svg</t>
+          <t>https://logos.hunter.io/sobaka.ru</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/d/db/Forbes_logo.svg</t>
+          <t>https://logos.hunter.io/forbes.ru</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>https://stroygaz.ru/upload/uf/e61/oekrgwiovsiba5ajvv6147lsauedss2g.webp</t>
+          <t>https://logos.hunter.io/stroygaz.ru</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>https://regnum.ru/main_logo.svg</t>
+          <t>https://logos.hunter.io/regnum.ru</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>https://topcor.ru/templates/topcor/images/logo.png</t>
+          <t>https://logos.hunter.io/topcor.ru</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>https://sfera.fm/assets/media/logo/logo_sfera_header.png</t>
+          <t>https://logos.hunter.io/sfera.fm</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7371,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>https://brl.mk.ru/media/mkru2020/img/mk-logo.svg</t>
+          <t>https://logos.hunter.io/brl.mk.ru</t>
         </is>
       </c>
     </row>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>https://novate.ru/img/logo.svg</t>
+          <t>https://logos.hunter.io/novate.ru</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7505,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>https://static.tildacdn.com/tild3930-3036-4536-a464-363733353938/BCB_logo_1.svg</t>
+          <t>https://logos.hunter.io/beautycarteblanche.ru</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7572,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://www.vokrug.tv/images/logo-new.svg</t>
+          <t>https://logos.hunter.io/vokrug.tv</t>
         </is>
       </c>
     </row>
@@ -7639,7 +7639,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/vokrugsveta/8b7f3beb.svg</t>
+          <t>https://logos.hunter.io/vokrugsveta.ru</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/woman/2cb6624f.svg</t>
+          <t>https://logos.hunter.io/oman.ru</t>
         </is>
       </c>
     </row>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/wday/2cb6624f.svg</t>
+          <t>https://logos.hunter.io/day.ru</t>
         </is>
       </c>
     </row>
@@ -7840,7 +7840,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://thegirl.ru/public/sprites/thegirl/e5cb1e72ce8b.svg</t>
+          <t>https://logos.hunter.io/thegirl.ru</t>
         </is>
       </c>
     </row>
@@ -7907,7 +7907,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/starhit/500f077c.svg</t>
+          <t>https://logos.hunter.io/starhit.ru</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/parents/b1a1d258.svg</t>
+          <t>https://logos.hunter.io/parents.ru</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8041,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/mcmaison/2cb6624f.svg</t>
+          <t>https://logos.hunter.io/mydecor.ru</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/doctorpiter/e4197781.svg</t>
+          <t>https://logos.hunter.io/doctorpiter.ru</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/wday/2cb6624f.svg</t>
+          <t>https://logos.hunter.io/the-day.ru</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/dist/maxim/f8d1d209.svg</t>
+          <t>https://logos.hunter.io/maximonline.ru</t>
         </is>
       </c>
     </row>
@@ -8309,7 +8309,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://cdn.hsmedia.ru/ump-webapp-public/dist/client/assets/psychologies_lg_bg-light-DG40Nryg.svg</t>
+          <t>https://logos.hunter.io/psychologies.ru</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8376,7 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>https://www.fashiontime.ru/bitrix/templates/ft.v3/images/logo.png</t>
+          <t>https://logos.hunter.io/fashiontime.ru</t>
         </is>
       </c>
     </row>
@@ -8443,7 +8443,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://oane.ws/templates/oane_new/logo-old.png</t>
+          <t>https://logos.hunter.io/oane.ws</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://terrnews.com/templates/Hint-utf8/images/logo66.png</t>
+          <t>https://logos.hunter.io/terrnews.com</t>
         </is>
       </c>
     </row>
@@ -8577,7 +8577,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://kadara.ru/wp-content/uploads/2019/12/kadara-logo.png</t>
+          <t>https://logos.hunter.io/kadara.ru</t>
         </is>
       </c>
     </row>
@@ -8644,7 +8644,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://monavista.ru/templates/newshub/images/logo-old.png</t>
+          <t>https://logos.hunter.io/monavista.ru</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://vestnik.net/images/logo_in_html.png</t>
+          <t>https://logos.hunter.io/vestnik.net</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://nvspost.ru/templates/lifewatcher/images/logo3.png</t>
+          <t>https://logos.hunter.io/nvspost.ru</t>
         </is>
       </c>
     </row>
@@ -8845,7 +8845,7 @@
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/6/68/K_Pravda_Logo_Modern.svg</t>
+          <t>https://logos.hunter.io/spb.kp.ru</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/6/68/K_Pravda_Logo_Modern.svg</t>
+          <t>https://logos.hunter.io/belarus.kp.ru</t>
         </is>
       </c>
     </row>
@@ -9046,7 +9046,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>https://news-24.ru/wp-content/uploads/2025/01/logon24.png</t>
+          <t>https://logos.hunter.io/news-24.ru</t>
         </is>
       </c>
     </row>
@@ -9113,7 +9113,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://smi24.news/wp-content/uploads/2024/12/group-158-1.svg</t>
+          <t>https://logos.hunter.io/smi24.news</t>
         </is>
       </c>
     </row>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://www.frequentflyers.ru/wp-content/uploads/2015/10/fflogo6.png</t>
+          <t>https://logos.hunter.io/frequentflyers.ru</t>
         </is>
       </c>
     </row>
@@ -9649,7 +9649,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://adindex.ru/assets/img/logo-adindex.svg</t>
+          <t>https://logos.hunter.io/adindex.ru</t>
         </is>
       </c>
     </row>
@@ -9716,7 +9716,7 @@
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://static.tildacdn.com/tild3938-6436-4639-b565-343838653436/Logo.svg</t>
+          <t>https://logos.hunter.io/artagmag.ru</t>
         </is>
       </c>
     </row>
@@ -9783,7 +9783,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://img.artlebedev.ru/everything/sport24/identity/media/icons/s24_port.svg</t>
+          <t>https://logos.hunter.io/sport24.ru</t>
         </is>
       </c>
     </row>
@@ -9850,7 +9850,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://prufy.ru/images/reg/prufy.ru.svg</t>
+          <t>https://logos.hunter.io/prufy.ru</t>
         </is>
       </c>
     </row>
@@ -9984,7 +9984,7 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://www.moneytimes.ru/images/moneytimes-logo.png</t>
+          <t>https://logos.hunter.io/moneytimes.ru</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://english.pravda.ru/pix/logo_white.png</t>
+          <t>https://logos.hunter.io/english.pravda.ru</t>
         </is>
       </c>
     </row>
@@ -10118,7 +10118,7 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>https://www.medpulse.ru/image/upload/logo512.jpg</t>
+          <t>https://logos.hunter.io/medpulse.ru</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10185,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>https://www.newsinfo.ru/images/newsinfo-logo.png</t>
+          <t>https://logos.hunter.io/newsinfo.ru</t>
         </is>
       </c>
     </row>
@@ -10252,7 +10252,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.politonline.ru/assets/logo-5-4679515ece2fdfeb4567553a15565643.png</t>
+          <t>https://logos.hunter.io/politonline.ru</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://www.yoki.ru/images/yoki-logo.png</t>
+          <t>https://logos.hunter.io/yoki.ru</t>
         </is>
       </c>
     </row>
@@ -10453,7 +10453,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>https://www.ecosever.ru/images/ecosever-logo.png</t>
+          <t>https://logos.hunter.io/ecosever.ru</t>
         </is>
       </c>
     </row>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://www.nationaljournal.ru/pix/nationaljournal-logo.png</t>
+          <t>https://logos.hunter.io/nationaljournal.ru</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://www.rusday.com/pix/rusday-logo.png</t>
+          <t>https://logos.hunter.io/rusday.com</t>
         </is>
       </c>
     </row>
@@ -10654,7 +10654,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://www.electorat.info/pix/electorat-logo.png</t>
+          <t>https://logos.hunter.io/electorat.info</t>
         </is>
       </c>
     </row>
@@ -10721,7 +10721,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://www.mostimes.com/images/mostimes-logo.png</t>
+          <t>https://logos.hunter.io/mostimes.com</t>
         </is>
       </c>
     </row>
@@ -10788,7 +10788,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>https://www.pora.ru/images/logo.png</t>
+          <t>https://logos.hunter.io/pora.ru</t>
         </is>
       </c>
     </row>
@@ -10855,7 +10855,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>https://www.glavtema.ru/pix/glavtema-logo.png</t>
+          <t>https://logos.hunter.io/glavtema.ru</t>
         </is>
       </c>
     </row>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>https://www.prbn.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/prbn.ru</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>https://www.bigness.ru/pix/logo.gif</t>
+          <t>https://logos.hunter.io/bigness.ru</t>
         </is>
       </c>
     </row>
@@ -11056,7 +11056,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>https://www.militarytimes.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/militarytimes.ru</t>
         </is>
       </c>
     </row>
@@ -11123,7 +11123,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>https://www.fizcultprivet.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/fizcultprivet.ru</t>
         </is>
       </c>
     </row>
@@ -11190,7 +11190,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>https://www.poplawok.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/poplawok.ru</t>
         </is>
       </c>
     </row>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>https://www.autokolonka.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/autokolonka.ru</t>
         </is>
       </c>
     </row>
@@ -11324,7 +11324,7 @@
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>https://www.repairshome.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/repairshome.ru</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11391,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>https://www.dailyshow.ru/images/dailyshow-logo.gif</t>
+          <t>https://logos.hunter.io/dailyshow.ru</t>
         </is>
       </c>
     </row>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>https://www.missus.ru/pix/logo.gif</t>
+          <t>https://logos.hunter.io/missus.ru</t>
         </is>
       </c>
     </row>
@@ -11525,7 +11525,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>https://www.bigcaucasus.com/pix/smalllogo.jpg</t>
+          <t>https://logos.hunter.io/bigcaucasus.com</t>
         </is>
       </c>
     </row>
@@ -11592,7 +11592,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>https://www.georgiatimes.info/images/georgiatimes-logo.jpg</t>
+          <t>https://logos.hunter.io/georgiatimes.info</t>
         </is>
       </c>
     </row>
@@ -11659,7 +11659,7 @@
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>https://www.pravda.ru/pix/logo600_60.png</t>
+          <t>https://logos.hunter.io/pravda.ru</t>
         </is>
       </c>
     </row>
@@ -11726,7 +11726,7 @@
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>https://aviation21.ru/wp-content/uploads/2017/03/logo-1.png</t>
+          <t>https://logos.hunter.io/aviation21.ru</t>
         </is>
       </c>
     </row>
@@ -11860,7 +11860,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>https://asninfo.ru/images/logo.png</t>
+          <t>https://logos.hunter.io/asninfo.ru</t>
         </is>
       </c>
     </row>
@@ -11927,7 +11927,7 @@
       </c>
       <c r="M171" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/2/24/TV78logo.svg</t>
+          <t>https://logos.hunter.io/78.ru</t>
         </is>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/6/67/Logo_of_Russian_magazine_The_Voice.svg</t>
+          <t>https://logos.hunter.io/thevoicemag.ru</t>
         </is>
       </c>
     </row>
@@ -12061,7 +12061,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>https://moskvichmag.ru/wp-content/themes/moskmag-new/assets/img/svg/mm-xl-logo.svg</t>
+          <t>https://logos.hunter.io/moskvichmag.ru</t>
         </is>
       </c>
     </row>
@@ -12128,7 +12128,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/f/f1/RBK_logo.svg</t>
+          <t>https://logos.hunter.io/rbc.ru</t>
         </is>
       </c>
     </row>
@@ -12195,7 +12195,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>https://moslenta.ru/favicon.svg</t>
+          <t>https://logos.hunter.io/moslenta.ru</t>
         </is>
       </c>
     </row>
@@ -12262,7 +12262,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>https://kapital.kz/logo.png</t>
+          <t>https://logos.hunter.io/kapital.kz</t>
         </is>
       </c>
     </row>
@@ -12329,7 +12329,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>https://lsm.kz/static/img/logo.png</t>
+          <t>https://logos.hunter.io/lsm.kz</t>
         </is>
       </c>
     </row>
@@ -12396,7 +12396,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>https://newsmaker.md/wp-content/uploads/2019/01/logo_square.jpg</t>
+          <t>https://logos.hunter.io/newsmaker.md</t>
         </is>
       </c>
     </row>
@@ -12463,7 +12463,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>https://cdn-1.aki.kg/st_akipress/logo_wide_300x48.png</t>
+          <t>https://logos.hunter.io/akipress.org</t>
         </is>
       </c>
     </row>
@@ -12530,7 +12530,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>https://24.kg/assets/39aedacb/images/logo.png</t>
+          <t>https://logos.hunter.io/24.kg</t>
         </is>
       </c>
     </row>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>https://noi.md/images/logo_noi_blue.jpg</t>
+          <t>https://logos.hunter.io/noi.md</t>
         </is>
       </c>
     </row>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>https://www.uzdaily.uz/static/web/files/logo.258d31191858.svg</t>
+          <t>https://logos.hunter.io/uzdaily.uz</t>
         </is>
       </c>
     </row>
@@ -12731,7 +12731,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>https://www.inform.kz/static/img/favicon.svg</t>
+          <t>https://logos.hunter.io/inform.kz</t>
         </is>
       </c>
     </row>
@@ -12798,7 +12798,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>https://remedium.ru/upload/medialibrary/43b/Remedium-logo-2019-MAIN.png</t>
+          <t>https://logos.hunter.io/remedium.ru</t>
         </is>
       </c>
     </row>
@@ -12865,7 +12865,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>https://medvestnik.ru/apps/mv/assets/cache/images/c7aa52eecd.svg</t>
+          <t>https://logos.hunter.io/medvestnik.ru</t>
         </is>
       </c>
     </row>
@@ -12932,7 +12932,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>https://incrussia.ru/wp-content/themes/inc/img/ink_logo_space.svg</t>
+          <t>https://logos.hunter.io/incrussia.ru</t>
         </is>
       </c>
     </row>
@@ -12999,7 +12999,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>https://apptractor.ru/wp-content/uploads/2025/10/logowebp-1.webp</t>
+          <t>https://logos.hunter.io/apptractor.ru</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>https://investfuture.ru/static/logo.png</t>
+          <t>https://logos.hunter.io/investfuture.ru</t>
         </is>
       </c>
     </row>
@@ -13133,7 +13133,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/commons/f/f3/Logo-onliner-by.png</t>
+          <t>https://logos.hunter.io/onliner.by</t>
         </is>
       </c>
     </row>
@@ -13200,7 +13200,7 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>https://bits.media/local/templates/bits.media/images/bits4.png</t>
+          <t>https://logos.hunter.io/bits.media</t>
         </is>
       </c>
     </row>
@@ -13267,7 +13267,7 @@
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>https://telegraf.news/_astro/logo_black.hKlVZoUa.svg</t>
+          <t>https://logos.hunter.io/telegraf.news</t>
         </is>
       </c>
     </row>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>https://liter.kz/build/images/liter-logo-news.png</t>
+          <t>https://logos.hunter.io/liter.kz</t>
         </is>
       </c>
     </row>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>https://orda.kz/img/logo_d.svg</t>
+          <t>https://logos.hunter.io/orda.kz</t>
         </is>
       </c>
     </row>
@@ -13468,7 +13468,7 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>https://dcjournal.ru/theme/codirf/images/h-logo6.png</t>
+          <t>https://logos.hunter.io/dcjournal.ru</t>
         </is>
       </c>
     </row>
@@ -13535,7 +13535,7 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>https://telecombloger.ru/wp-content/uploads/2024/12/Logo.png</t>
+          <t>https://logos.hunter.io/telecombloger.ru</t>
         </is>
       </c>
     </row>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>https://urbc.ru/templates/Default/images/logo.svg</t>
+          <t>https://logos.hunter.io/urbc.ru</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>https://upload.wikimedia.org/wikipedia/ru/9/9d/%D0%9B%D0%BE%D0%B3%D0%BE%D1%82%D0%B8%D0%BF_Haqqin.az.svg</t>
+          <t>https://logos.hunter.io/haqqin.az</t>
         </is>
       </c>
     </row>
@@ -13736,7 +13736,7 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>https://www.mosregion.info/wp-content/uploads/2024/09/mosregion_logo.png</t>
+          <t>https://logos.hunter.io/mosregion.info</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13803,7 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>https://www.sila-rf.ru/wp-content/uploads/2022/02/sila-rf.png</t>
+          <t>https://logos.hunter.io/sila-rf.ru</t>
         </is>
       </c>
     </row>
@@ -13870,7 +13870,7 @@
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>https://www.sibmedia.ru/wp-content/uploads/2024/07/sibmedia_logo.png</t>
+          <t>https://logos.hunter.io/sibmedia.ru</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>https://www.ladys.media/wp-content/themes/ladys/images/logos/logo_desktop.svg</t>
+          <t>https://logos.hunter.io/ladys.media</t>
         </is>
       </c>
     </row>
@@ -14004,7 +14004,7 @@
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>https://www.socialinform.ru/wp-content/uploads/2024/02/socnews_logo-1.png</t>
+          <t>https://logos.hunter.io/socialinform.ru</t>
         </is>
       </c>
     </row>
@@ -14071,7 +14071,7 @@
       </c>
       <c r="M203" t="inlineStr">
         <is>
-          <t>https://www.myeconomy.ru/wp-content/uploads/2024/11/economy-logo.png</t>
+          <t>https://logos.hunter.io/myeconomy.ru</t>
         </is>
       </c>
     </row>
@@ -14138,7 +14138,7 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>https://www.ecopravda.ru/wp-content/uploads/2022/07/Group-210.jpg</t>
+          <t>https://logos.hunter.io/ecopravda.ru</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14205,7 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>https://medzdrav.info/wp-content/uploads/2024/01/logo_header.svg</t>
+          <t>https://logos.hunter.io/medzdrav.info</t>
         </is>
       </c>
     </row>
@@ -14272,7 +14272,7 @@
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>https://today.ua/svg/logo.svg</t>
+          <t>https://logos.hunter.io/today.ua</t>
         </is>
       </c>
     </row>
@@ -14339,7 +14339,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>https://beautyhunter.ru/attachments/Image/bhlogo36.png</t>
+          <t>https://logos.hunter.io/beautyhunter.ru</t>
         </is>
       </c>
     </row>
@@ -14406,7 +14406,7 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>https://informator.ua/images/logo.svg</t>
+          <t>https://logos.hunter.io/informator.ua</t>
         </is>
       </c>
     </row>
@@ -14473,7 +14473,7 @@
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t>https://itechua.com/wp-content/uploads/2024/08/itechua-logo.png</t>
+          <t>https://logos.hunter.io/itechua.com</t>
         </is>
       </c>
     </row>
@@ -14540,7 +14540,7 @@
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t>https://mignews.ua/static/img/logo_ua.png</t>
+          <t>https://logos.hunter.io/mignews.ua</t>
         </is>
       </c>
     </row>
@@ -14607,7 +14607,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>https://www.it-world.ru/local/templates/.default/img/logo/logo_s1.svg</t>
+          <t>https://logos.hunter.io/it-world.ru</t>
         </is>
       </c>
     </row>
@@ -14675,7 +14675,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>https://gazeta.ua/images/svg/gazeta.svg</t>
+          <t>https://logos.hunter.io/gazeta.ua</t>
         </is>
       </c>
     </row>

</xml_diff>